<commit_message>
change in audit nature
</commit_message>
<xml_diff>
--- a/executive/companies/company_bulk_template.xlsx
+++ b/executive/companies/company_bulk_template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\OneDrive\Desktop\Download\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp-check\htdocs\mis\executive\companies\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D558A46D-503F-4A57-938F-648B9053D16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4575"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Companies" sheetId="1" r:id="rId1"/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>Company Name *</t>
   </si>
@@ -58,27 +59,12 @@
     <t>Address</t>
   </si>
   <si>
-    <t>Private Limited</t>
-  </si>
-  <si>
     <t>D1</t>
   </si>
   <si>
-    <t>Trading</t>
-  </si>
-  <si>
-    <t>Public Limited</t>
-  </si>
-  <si>
     <t>D2</t>
   </si>
   <si>
-    <t>Service</t>
-  </si>
-  <si>
-    <t>Partnership</t>
-  </si>
-  <si>
     <t>D3</t>
   </si>
   <si>
@@ -106,9 +92,6 @@
     <t>3. company_type / branch_name / industry_name</t>
   </si>
   <si>
-    <t>Sole Proprietorship</t>
-  </si>
-  <si>
     <t>D4</t>
   </si>
   <si>
@@ -118,9 +101,6 @@
     <t xml:space="preserve">   must match values in this sheet exactly.</t>
   </si>
   <si>
-    <t>NGO/INGO</t>
-  </si>
-  <si>
     <t>Finance</t>
   </si>
   <si>
@@ -136,18 +116,12 @@
     <t>5. Provide company_code to UPDATE existing.</t>
   </si>
   <si>
-    <t>Government</t>
-  </si>
-  <si>
     <t>IT</t>
   </si>
   <si>
     <t>6. PAN must be 10 digits and unique.</t>
   </si>
   <si>
-    <t>Others</t>
-  </si>
-  <si>
     <t>Healthcare</t>
   </si>
   <si>
@@ -173,13 +147,58 @@
   </si>
   <si>
     <t>Kawosoti Branch</t>
+  </si>
+  <si>
+    <t>Pvt Ltd</t>
+  </si>
+  <si>
+    <t>Public Company</t>
+  </si>
+  <si>
+    <t>partnership</t>
+  </si>
+  <si>
+    <t>NPO</t>
+  </si>
+  <si>
+    <t>Samuha</t>
+  </si>
+  <si>
+    <t>JV</t>
+  </si>
+  <si>
+    <t>Proprietorship</t>
+  </si>
+  <si>
+    <t>AGRO-Livestock Farming</t>
+  </si>
+  <si>
+    <t>AGRO-Plant Farming</t>
+  </si>
+  <si>
+    <t>Automobile Industry</t>
+  </si>
+  <si>
+    <t>Dairy Industry</t>
+  </si>
+  <si>
+    <t>FMCG-Wholesaler</t>
+  </si>
+  <si>
+    <t>Furniture Suppliers</t>
+  </si>
+  <si>
+    <t>Hospitality Industry</t>
+  </si>
+  <si>
+    <t>INGO/NGO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +236,24 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -286,7 +323,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -300,7 +337,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -310,9 +346,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -321,6 +354,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -624,7 +664,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -679,172 +719,167 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="5" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="1:12" s="5" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-    </row>
-    <row r="4" spans="1:12" s="5" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="6"/>
-    </row>
-    <row r="5" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-    </row>
-    <row r="7" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="17" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="18" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="19" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="20" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="22" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="23" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="24" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="25" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="26" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="27" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="30" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="31" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="32" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="61" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="62" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="63" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="64" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="65" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="66" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="67" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="68" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="69" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="70" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="71" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="72" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="73" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="74" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="76" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="78" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="79" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="80" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="81" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="82" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="83" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="84" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="85" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="86" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="87" s="5" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+    </row>
+    <row r="17" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="18" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="19" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="20" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="22" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="23" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="24" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="25" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="26" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="28" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="29" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="30" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="31" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="32" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="33" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="35" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="36" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="84" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="85" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="86" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="87" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>'Valid Values'!$C$2:$C$11</xm:f>
-          </x14:formula1>
-          <xm:sqref>H2:H48</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>'Valid Values'!$B$2:$B$5</xm:f>
           </x14:formula1>
           <xm:sqref>G1:G1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>'Valid Values'!$E$2:$E$4</xm:f>
           </x14:formula1>
           <xm:sqref>F2:F1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>'Valid Values'!$A$2:$A$9</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>'Valid Values'!$C$2:$C$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>H3:H48</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DCA9036F-7A94-48BF-82EA-7CAA4D1C5E03}">
+          <x14:formula1>
+            <xm:f>'Valid Values'!$C$2:$C$16</xm:f>
+          </x14:formula1>
+          <xm:sqref>H2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -853,8 +888,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="30" customWidth="1"/>
@@ -864,147 +899,173 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>23</v>
+        <v>17</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>47</v>
+      <c r="E2" s="9" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>50</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>50</v>
+        <v>21</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>49</v>
+        <v>22</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>30</v>
+        <v>23</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>24</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>29</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>36</v>
+        <v>46</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>52</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>39</v>
+        <v>47</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C10" s="3" t="s">
-        <v>44</v>
+      <c r="C10" s="12" t="s">
+        <v>53</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C11" s="4" t="s">
-        <v>41</v>
+      <c r="C11" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>46</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C12" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C13" s="12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C14" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C15" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="12" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>